<commit_message>
Complete Procurement KB export, add agent and procurement indexes
- All 11 Procurement Knowledge Base policy pages exported in wiki Order.
- Index READMEs for agents/ and procurement-knowledge-base/, noting that the
  Questionnaire Autofill Agent page returns 404 from the integration.
- Calculator README tab documents why formula cells ship without cached values
  and how the engine was verified instead.

Co-Authored-By: Claude Opus 5 <noreply@anthropic.com>
Claude-Session: https://claude.ai/code/session_01B47DUcQnhymW8ZZ9KdGGwV
</commit_message>
<xml_diff>
--- a/notion-exports/April_DIY_Pricing_2.0_Calculator.xlsx
+++ b/notion-exports/April_DIY_Pricing_2.0_Calculator.xlsx
@@ -121,7 +121,7 @@
   <cellStyleXfs count="1">
     <xf numFmtId="0" fontId="0" fillId="0" borderId="0"/>
   </cellStyleXfs>
-  <cellXfs count="30">
+  <cellXfs count="31">
     <xf numFmtId="0" fontId="0" fillId="0" borderId="0" pivotButton="0" quotePrefix="0" xfId="0"/>
     <xf numFmtId="0" fontId="1" fillId="0" borderId="0" pivotButton="0" quotePrefix="0" xfId="0"/>
     <xf numFmtId="0" fontId="2" fillId="0" borderId="0" pivotButton="0" quotePrefix="0" xfId="0"/>
@@ -154,6 +154,9 @@
     <xf numFmtId="168" fontId="6" fillId="3" borderId="1" pivotButton="0" quotePrefix="0" xfId="0"/>
     <xf numFmtId="168" fontId="6" fillId="0" borderId="1" pivotButton="0" quotePrefix="0" xfId="0"/>
     <xf numFmtId="0" fontId="5" fillId="0" borderId="1" applyAlignment="1" pivotButton="0" quotePrefix="0" xfId="0">
+      <alignment vertical="top" wrapText="1"/>
+    </xf>
+    <xf numFmtId="0" fontId="2" fillId="0" borderId="0" applyAlignment="1" pivotButton="0" quotePrefix="0" xfId="0">
       <alignment vertical="top" wrapText="1"/>
     </xf>
   </cellXfs>
@@ -521,7 +524,7 @@
     <outlinePr summaryBelow="1" summaryRight="1"/>
     <pageSetUpPr/>
   </sheetPr>
-  <dimension ref="B2:C37"/>
+  <dimension ref="B2:C40"/>
   <sheetFormatPr baseColWidth="8" defaultRowHeight="15"/>
   <cols>
     <col width="3" customWidth="1" min="1" max="1"/>
@@ -781,6 +784,20 @@
       <c r="C37" s="5" t="inlineStr">
         <is>
           <t>- DIY unit cost: need fully loaded cost per filing to confirm the $7.00 floor clears the margin target.</t>
+        </is>
+      </c>
+    </row>
+    <row r="39">
+      <c r="B39" s="3" t="inlineStr">
+        <is>
+          <t>Recalculation note</t>
+        </is>
+      </c>
+    </row>
+    <row r="40" ht="70" customHeight="1">
+      <c r="C40" s="30" t="inlineStr">
+        <is>
+          <t>Formula cells carry no cached values: this workbook was written programmatically and LibreOffice was unavailable in the build environment to pre-compute them. Excel, Google Sheets and Numbers all recalculate on open, so the grids fill in as soon as you open the file. The engine itself was verified independently: it reproduces every cell of the memo's published rate matrix and blended-rate grid (see the variance note above for the single $0.10 rounding tie).</t>
         </is>
       </c>
     </row>

</xml_diff>